<commit_message>
refactor: add multiple sheet support and refactor project
</commit_message>
<xml_diff>
--- a/src/main/resources/test.xlsx
+++ b/src/main/resources/test.xlsx
@@ -1,12 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tmehmetkadioglu\Desktop\file-reader\src\main\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCD7CA6-2300-4558-A613-57BA14C764F6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="dt" sheetId="1" r:id="rId4"/>
+    <sheet name="dt" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="31TbsXSoahfDFGtgNQeLRULbkl1I0piGUexVKPFHETs="/>
@@ -16,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -67,36 +77,61 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>2025-07-02T14:22:54.737232300+03:00</t>
+  </si>
+  <si>
+    <t>2025-07-02T11:25:53.819050600Z</t>
+  </si>
+  <si>
+    <t>2025-07-02T11:25:53.819050Z</t>
+  </si>
+  <si>
+    <t>2025-07-02T11:25:53.819Z</t>
+  </si>
+  <si>
+    <t>2025-07-03T10:15:30Z</t>
+  </si>
+  <si>
+    <t>2025-07-03T10:15:30+03:00</t>
+  </si>
+  <si>
+    <t>2025-07-03T10:15:30.123Z</t>
+  </si>
+  <si>
+    <t>2025-07-03T10:15:30.123456+03:00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="d.m.yyyy hh:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="d-m-yyyy"/>
+    <numFmt numFmtId="164" formatCode="d\.m\.yyyy\ hh:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="d\-m\-yyyy"/>
     <numFmt numFmtId="166" formatCode="d/m/yyyy"/>
-    <numFmt numFmtId="167" formatCode="yyyy/m/d hh:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="yyyy/m/d\ hh:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="9.0"/>
+      <sz val="9"/>
       <color rgb="FF000000"/>
       <name val="&quot;Google Sans Mono&quot;"/>
     </font>
@@ -106,7 +141,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -116,62 +151,71 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="12">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="167" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -361,34 +405,37 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
-    <pageSetUpPr/>
+    <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <dimension ref="A1:O1000"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="10.5"/>
-    <col customWidth="1" min="2" max="2" width="5.75"/>
-    <col customWidth="1" min="3" max="3" width="13.13"/>
-    <col customWidth="1" min="4" max="4" width="17.63"/>
-    <col customWidth="1" min="5" max="5" width="8.38"/>
-    <col customWidth="1" min="6" max="6" width="9.63"/>
-    <col customWidth="1" min="7" max="7" width="13.88"/>
-    <col customWidth="1" min="8" max="8" width="10.63"/>
-    <col customWidth="1" min="9" max="9" width="7.25"/>
-    <col customWidth="1" min="10" max="10" width="9.0"/>
-    <col customWidth="1" min="11" max="11" width="8.38"/>
-    <col customWidth="1" min="12" max="12" width="5.5"/>
-    <col customWidth="1" min="13" max="13" width="8.75"/>
-    <col customWidth="1" min="14" max="15" width="8.38"/>
-    <col customWidth="1" min="16" max="26" width="8.0"/>
+    <col min="1" max="1" width="10.453125" customWidth="1"/>
+    <col min="2" max="2" width="5.7265625" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="4" max="4" width="41.81640625" customWidth="1"/>
+    <col min="5" max="5" width="34.7265625" customWidth="1"/>
+    <col min="6" max="6" width="35.453125" customWidth="1"/>
+    <col min="7" max="7" width="13.81640625" customWidth="1"/>
+    <col min="8" max="8" width="10.54296875" customWidth="1"/>
+    <col min="9" max="9" width="7.26953125" customWidth="1"/>
+    <col min="10" max="10" width="9" customWidth="1"/>
+    <col min="11" max="11" width="8.453125" customWidth="1"/>
+    <col min="12" max="12" width="5.453125" customWidth="1"/>
+    <col min="13" max="13" width="8.7265625" customWidth="1"/>
+    <col min="14" max="15" width="8.453125" customWidth="1"/>
+    <col min="16" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12.75" customHeight="1">
+    <row r="1" spans="1:15" ht="12.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -425,7 +472,7 @@
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" ht="12.75" customHeight="1">
+    <row r="2" spans="1:15" ht="12.75" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -435,11 +482,11 @@
       <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="4">
-        <v>45242.530960648146</v>
-      </c>
-      <c r="E2" s="4">
-        <v>45242.530960648146</v>
+      <c r="D2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>18</v>
       </c>
       <c r="F2" s="4">
         <v>45242.530960648146</v>
@@ -448,13 +495,13 @@
         <v>10</v>
       </c>
       <c r="H2" s="5">
-        <v>35646.0</v>
+        <v>35646</v>
       </c>
       <c r="I2" s="5">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="J2" s="5">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
@@ -462,9 +509,9 @@
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
     </row>
-    <row r="3" ht="12.75" customHeight="1">
+    <row r="3" spans="1:15" ht="12.75" customHeight="1">
       <c r="A3" s="6">
-        <v>45242.0</v>
+        <v>45242</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>13</v>
@@ -472,26 +519,26 @@
       <c r="C3" s="5">
         <v>571.39</v>
       </c>
-      <c r="D3" s="7">
-        <v>45242.530960648146</v>
-      </c>
-      <c r="E3" s="7">
-        <v>45242.530960648146</v>
+      <c r="D3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>19</v>
       </c>
       <c r="F3" s="7">
         <v>45242.530960648146</v>
       </c>
       <c r="G3" s="6">
-        <v>45242.0</v>
+        <v>45242</v>
       </c>
       <c r="H3" s="5">
-        <v>12132.0</v>
+        <v>12132</v>
       </c>
       <c r="I3" s="5">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="J3" s="5">
-        <v>87.0</v>
+        <v>87</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
@@ -499,9 +546,9 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
     </row>
-    <row r="4" ht="12.75" customHeight="1">
+    <row r="4" spans="1:15" ht="12.75" customHeight="1">
       <c r="A4" s="8">
-        <v>45242.0</v>
+        <v>45242</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>14</v>
@@ -509,24 +556,24 @@
       <c r="C4" s="5">
         <v>2.17</v>
       </c>
-      <c r="D4" s="9">
-        <v>45240.39913194445</v>
-      </c>
-      <c r="E4" s="9">
-        <v>45240.39913194445</v>
+      <c r="D4" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>20</v>
       </c>
       <c r="F4" s="9">
-        <v>45240.39913194445</v>
+        <v>45240.399131944447</v>
       </c>
       <c r="G4" s="8">
-        <v>45242.0</v>
+        <v>45242</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="5">
-        <v>65.0</v>
+        <v>65</v>
       </c>
       <c r="J4" s="5">
-        <v>98.0</v>
+        <v>98</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
@@ -534,7 +581,7 @@
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
     </row>
-    <row r="5" ht="12.75" customHeight="1">
+    <row r="5" spans="1:15" ht="12.75" customHeight="1">
       <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
@@ -542,9 +589,11 @@
         <v>15</v>
       </c>
       <c r="C5" s="10">
-        <v>24893.0</v>
-      </c>
-      <c r="D5" s="3"/>
+        <v>24893</v>
+      </c>
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
@@ -559,11 +608,13 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
     </row>
-    <row r="6" ht="12.75" customHeight="1">
+    <row r="6" spans="1:15" ht="12.75" customHeight="1">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -576,7 +627,7 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
     </row>
-    <row r="7" ht="12.75" customHeight="1">
+    <row r="7" spans="1:15" ht="12.75" customHeight="1">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -593,7 +644,7 @@
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
     </row>
-    <row r="8" ht="12.75" customHeight="1">
+    <row r="8" spans="1:15" ht="12.75" customHeight="1">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -610,7 +661,7 @@
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
     </row>
-    <row r="9" ht="12.75" customHeight="1">
+    <row r="9" spans="1:15" ht="12.75" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -630,7 +681,7 @@
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
     </row>
-    <row r="10" ht="12.75" customHeight="1">
+    <row r="10" spans="1:15" ht="12.75" customHeight="1">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -647,7 +698,7 @@
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
     </row>
-    <row r="11" ht="12.75" customHeight="1">
+    <row r="11" spans="1:15" ht="12.75" customHeight="1">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -664,7 +715,7 @@
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
     </row>
-    <row r="12" ht="12.75" customHeight="1">
+    <row r="12" spans="1:15" ht="12.75" customHeight="1">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -681,7 +732,7 @@
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
     </row>
-    <row r="13" ht="12.75" customHeight="1">
+    <row r="13" spans="1:15" ht="12.75" customHeight="1">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -698,7 +749,7 @@
       <c r="N13" s="3"/>
       <c r="O13" s="3"/>
     </row>
-    <row r="14" ht="12.75" customHeight="1">
+    <row r="14" spans="1:15" ht="12.75" customHeight="1">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -715,7 +766,7 @@
       <c r="N14" s="3"/>
       <c r="O14" s="3"/>
     </row>
-    <row r="15" ht="12.75" customHeight="1">
+    <row r="15" spans="1:15" ht="12.75" customHeight="1">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -732,7 +783,7 @@
       <c r="N15" s="3"/>
       <c r="O15" s="3"/>
     </row>
-    <row r="16" ht="12.75" customHeight="1">
+    <row r="16" spans="1:15" ht="12.75" customHeight="1">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -749,7 +800,7 @@
       <c r="N16" s="3"/>
       <c r="O16" s="3"/>
     </row>
-    <row r="17" ht="12.75" customHeight="1">
+    <row r="17" spans="1:15" ht="12.75" customHeight="1">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -766,7 +817,7 @@
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
     </row>
-    <row r="18" ht="12.75" customHeight="1">
+    <row r="18" spans="1:15" ht="12.75" customHeight="1">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -783,7 +834,7 @@
       <c r="N18" s="3"/>
       <c r="O18" s="3"/>
     </row>
-    <row r="19" ht="12.75" customHeight="1">
+    <row r="19" spans="1:15" ht="12.75" customHeight="1">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -800,7 +851,7 @@
       <c r="N19" s="3"/>
       <c r="O19" s="3"/>
     </row>
-    <row r="20" ht="12.75" customHeight="1">
+    <row r="20" spans="1:15" ht="12.75" customHeight="1">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -817,7 +868,7 @@
       <c r="N20" s="3"/>
       <c r="O20" s="3"/>
     </row>
-    <row r="21" ht="12.75" customHeight="1">
+    <row r="21" spans="1:15" ht="12.75" customHeight="1">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -834,7 +885,7 @@
       <c r="N21" s="3"/>
       <c r="O21" s="3"/>
     </row>
-    <row r="22" ht="12.75" customHeight="1">
+    <row r="22" spans="1:15" ht="12.75" customHeight="1">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -851,7 +902,7 @@
       <c r="N22" s="3"/>
       <c r="O22" s="3"/>
     </row>
-    <row r="23" ht="12.75" customHeight="1">
+    <row r="23" spans="1:15" ht="12.75" customHeight="1">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -892,7 +943,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="24" ht="12.75" customHeight="1">
+    <row r="24" spans="1:15" ht="12.75" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -933,7 +984,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" ht="12.75" customHeight="1">
+    <row r="25" spans="1:15" ht="12.75" customHeight="1">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -974,13 +1025,13 @@
         <v>16</v>
       </c>
     </row>
-    <row r="26" ht="12.75" customHeight="1"/>
-    <row r="27" ht="12.75" customHeight="1"/>
-    <row r="28" ht="12.75" customHeight="1"/>
-    <row r="29" ht="12.75" customHeight="1"/>
-    <row r="30" ht="12.75" customHeight="1"/>
-    <row r="31" ht="12.75" customHeight="1"/>
-    <row r="32" ht="12.75" customHeight="1"/>
+    <row r="26" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="27" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="28" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="29" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="30" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="31" spans="1:15" ht="12.75" customHeight="1"/>
+    <row r="32" spans="1:15" ht="12.75" customHeight="1"/>
     <row r="33" ht="12.75" customHeight="1"/>
     <row r="34" ht="12.75" customHeight="1"/>
     <row r="35" ht="12.75" customHeight="1"/>
@@ -1950,9 +2001,72 @@
     <row r="999" ht="12.75" customHeight="1"/>
     <row r="1000" ht="12.75" customHeight="1"/>
   </sheetData>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Calibri,Regular"&amp;10</oddHeader>
+    <evenHeader>&amp;L&amp;"Calibri,Regular"&amp;10</evenHeader>
+    <firstHeader>&amp;L&amp;"Calibri,Regular"&amp;10</firstHeader>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2707659-A29A-4ACA-886A-09017AE2483F}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="12.5"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Calibri,Regular"&amp;10</oddHeader>
+    <evenHeader>&amp;L&amp;"Calibri,Regular"&amp;10</evenHeader>
+    <firstHeader>&amp;L&amp;"Calibri,Regular"&amp;10</firstHeader>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<WrappedLabelHistory xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns="http://www.boldonjames.com/2016/02/Classifier/internal/wrappedLabelHistory">
+  <Value>PD94bWwgdmVyc2lvbj0iMS4wIiBlbmNvZGluZz0idXMtYXNjaWkiPz48bGFiZWxIaXN0b3J5IHhtbG5zOnhzZD0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEiIHhtbG5zOnhzaT0iaHR0cDovL3d3dy53My5vcmcvMjAwMS9YTUxTY2hlbWEtaW5zdGFuY2UiIHhtbG5zPSJodHRwOi8vd3d3LmJvbGRvbmphbWVzLmNvbS8yMDE2LzAyL0NsYXNzaWZpZXIvaW50ZXJuYWwvbGFiZWxIaXN0b3J5Ij48aXRlbT48c2lzbCBzaXNsVmVyc2lvbj0iMCIgcG9saWN5PSIyYjQ5ODY3Yi1hY2UzLTQwOGEtYjdlNC02ZDJhMzkxOTVmYzYiIG9yaWdpbj0idXNlclNlbGVjdGVkIj48ZWxlbWVudCB1aWQ9ImlkX2NsYXNzaWZpY2F0aW9uX25vbmJ1c2luZXNzIiB2YWx1ZT0iIiB4bWxucz0iaHR0cDovL3d3dy5ib2xkb25qYW1lcy5jb20vMjAwOC8wMS9zaWUvaW50ZXJuYWwvbGFiZWwiIC8+PGVsZW1lbnQgdWlkPSIzM2QwZGQ4Zi02MjkxLTQ0ZTktOTBlOS1lOTNlOWU0MGQ3ZTkiIHZhbHVlPSIiIHhtbG5zPSJodHRwOi8vd3d3LmJvbGRvbmphbWVzLmNvbS8yMDA4LzAxL3NpZS9pbnRlcm5hbC9sYWJlbCIgLz48L3Npc2w+PFVzZXJOYW1lPkVQSUFTXG1laG1ldC5rYWRpb2dsdTwvVXNlck5hbWU+PERhdGVUaW1lPjIuMDcuMjAyNSAxMToyNDo1ODwvRGF0ZVRpbWU+PExhYmVsU3RyaW5nPlRhc25pZiBEJiN4MTMxOyYjeDE1RjsmI3gxMzE7LUtpJiN4MTVGO2lzZWwgVmVyaSBpJiN4RTc7ZXJtZXo8L0xhYmVsU3RyaW5nPjwvaXRlbT48L2xhYmVsSGlzdG9yeT4=</Value>
+</WrappedLabelHistory>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<sisl xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns="http://www.boldonjames.com/2008/01/sie/internal/label" sislVersion="0" policy="2b49867b-ace3-408a-b7e4-6d2a39195fc6" origin="userSelected">
+  <element uid="id_classification_nonbusiness" value=""/>
+  <element uid="33d0dd8f-6291-44e9-90e9-e93e9e40d7e9" value=""/>
+</sisl>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{109BB78A-B193-4175-AC39-F58EBD287718}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://www.boldonjames.com/2016/02/Classifier/internal/wrappedLabelHistory"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{490757D5-676C-4473-9B64-C56914DF29ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://www.boldonjames.com/2008/01/sie/internal/label"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor: add new cell processors support
</commit_message>
<xml_diff>
--- a/src/main/resources/test.xlsx
+++ b/src/main/resources/test.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tmehmetkadioglu\Desktop\file-reader\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCCD7CA6-2300-4558-A613-57BA14C764F6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1964E75E-498E-41FA-9D7E-32F471868D03}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="29">
   <si>
     <t>Date</t>
   </si>
@@ -101,6 +101,18 @@
   </si>
   <si>
     <t>2025-07-03T10:15:30.123456+03:00</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>testEnum</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>TEST2</t>
   </si>
 </sst>
 </file>
@@ -466,8 +478,12 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="K1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>26</v>
+      </c>
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
@@ -503,8 +519,12 @@
       <c r="J2" s="5">
         <v>65</v>
       </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
+      <c r="K2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>27</v>
+      </c>
       <c r="M2" s="3"/>
       <c r="N2" s="3"/>
       <c r="O2" s="3"/>
@@ -540,8 +560,12 @@
       <c r="J3" s="5">
         <v>87</v>
       </c>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
+      <c r="K3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
@@ -575,7 +599,9 @@
       <c r="J4" s="5">
         <v>98</v>
       </c>
-      <c r="K4" s="3"/>
+      <c r="K4" s="3" t="b">
+        <v>0</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -2063,7 +2089,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{490757D5-676C-4473-9B64-C56914DF29ED}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0CB3A69-CDB8-4FAC-AEFA-8538822918EB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
     <ds:schemaRef ds:uri="http://www.boldonjames.com/2008/01/sie/internal/label"/>

</xml_diff>